<commit_message>
database: English self-service guide for museums
</commit_message>
<xml_diff>
--- a/database/review_translations.xlsx
+++ b/database/review_translations.xlsx
@@ -532,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="14.45"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -572,7 +572,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Une cellule jaune qui porte le commentaire « Traduction automatique (DeepL) — à relire » n'a encore été relue par personne.</t>
+          <t>Une cellule jaune qui porte le commentaire « Traduction automatique (DeepL), à relire » n'a encore été relue par personne.</t>
         </is>
       </c>
     </row>
@@ -643,6 +643,68 @@
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">• Témoignages </t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>Read me (English)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Only the cells with a YELLOW background (columns fr, nl, en) are to be corrected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Do not change the id and source columns or the cells with a GREY background.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>A yellow cell with the comment "Machine translation (DeepL), to review" has not been reviewed by anyone yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Do not insert, delete or move rows, and do not rename the sheets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>The id column is the TRACES ID of the artwork (import_collection.py prints the IDs of your new artworks); in "Types d'objets" it is the ID of the object type.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Sheets: Types d'objets (object types), Questions, Descriptions, Description - Key words (keywords), Emotions,</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Transcriptions, Transcriptions Explications (explanations of the transcriptions), Témoignages (interviews), Titres (titles).</t>
         </is>
       </c>
     </row>

</xml_diff>